<commit_message>
One eligibility rule for registering
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-51_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-51_Test_Cases.xlsx
@@ -7,19 +7,18 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open Questions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC01" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC02" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC03" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC04" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC05" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC06" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC07" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC08" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC09" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC10" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC11" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC12" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC01" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC02" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC03" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC04" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC05" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC06" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC07" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC08" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC09" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC10" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC11" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC12" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1200,7 +1199,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC08</t>
+          <t>SPM-51-TC09</t>
         </is>
       </c>
     </row>
@@ -1213,12 +1212,12 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Test data loaded: `npm run fixtures:spm51` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM51 …' events, never anyone else's data).
-Logged in as Chua Mei Ling (chua.mei.ling@example.com / password123), an Attendee.
-Nothing is saved in this case.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="31" customHeight="1">
+Nothing is saved in this case.
+Start logged in as Daniel Tan (daniel.tan@connectsphere.com / password123), the coordinator of every 'SPM51 …' event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="125.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1226,7 +1225,10 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Browse Events' in the sidebar and open 'SPM51 Undated Talk'</t>
+          <t>1. Click 'All Events' in the sidebar and open 'SPM51 Planning Stage Forum'
+2. Note the event's reference (EVT- number) shown on the page
+3. Log out and log in as Chua Mei Ling (chua.mei.ling@example.com / password123), an Attendee
+4. Type /events/&lt;reference from step 2&gt; after the site address in the browser address bar (e.g. http://localhost:3000/events/&lt;reference from step 2&gt;) and press Enter</t>
         </is>
       </c>
     </row>
@@ -1238,11 +1240,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM51 Undated Talk (Confirmed, registration on, capacity 50, no opening or closing date)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Event: SPM51 Planning Stage Forum (Planning, registration on, open period) | Attendee: Chua Mei Ling</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1250,7 +1252,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The Registration card shows 'Opens: —' and 'Closes: —'. The 'Your registration' card says 'Registration dates haven't been set for this event.' and has no 'Register' button.</t>
+          <t>Step 1: The event page shows the 'Planning' status badge.
+Step 4: The page shows 'This event doesn't exist, or you don't have access to it.' and nothing about registering.</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1362,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC09</t>
+          <t>SPM-51-TC10</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1376,7 @@
         <is>
           <t>Test data loaded: `npm run fixtures:spm51` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM51 …' events, never anyone else's data).
 Nothing is saved in this case.
-Start logged in as Daniel Tan (daniel.tan@connectsphere.com / password123), the coordinator of every 'SPM51 …' event.</t>
+Start logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
         </is>
       </c>
     </row>
@@ -1385,9 +1388,9 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'All Events' in the sidebar and open 'SPM51 Planning Stage Forum'
+          <t>1. Click 'All Events' in the sidebar and open 'SPM51 Private Board Dinner'
 2. Note the event's reference (EVT- number) shown on the page
-3. Log out and log in as Chua Mei Ling (chua.mei.ling@example.com / password123), an Attendee
+3. Log out and log in as Marcus Yeo (marcus.yeo@example.com / password123), an Attendee
 4. Type /events/&lt;reference from step 2&gt; after the site address in the browser address bar (e.g. http://localhost:3000/events/&lt;reference from step 2&gt;) and press Enter</t>
         </is>
       </c>
@@ -1400,11 +1403,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM51 Planning Stage Forum (Planning, registration on, open period) | Attendee: Chua Mei Ling</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44.5" customHeight="1">
+          <t>Event: SPM51 Private Board Dinner (Confirmed, registration off) | Attendee: Marcus Yeo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1412,7 +1415,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The event page shows the 'Planning' status badge.
+          <t>Step 1: The event page shows the 'Confirmed' status badge and 'Registration: Not enabled for this event'.
 Step 4: The page shows 'This event doesn't exist, or you don't have access to it.' and nothing about registering.</t>
         </is>
       </c>
@@ -1522,11 +1525,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC10</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="98.5" customHeight="1">
+          <t>SPM-51-TC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="139" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1535,12 +1538,12 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Test data loaded: `npm run fixtures:spm51` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM51 …' events, never anyone else's data).
-Nothing is saved in this case.
-Start logged in as Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="125.5" customHeight="1">
+Logged in as Jocelyn Pang (jocelyn.pang@example.com / password123), an Attendee registered for 'SPM51 Last Seat Masterclass' and on the waiting list for 'SPM51 Sold Out Summit'. (The base seed may register her for other events too; those rows are listed as well.)
+Nothing is saved in this case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="31" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1548,10 +1551,8 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'All Events' in the sidebar and open 'SPM51 Private Board Dinner'
-2. Note the event's reference (EVT- number) shown on the page
-3. Log out and log in as Marcus Yeo (marcus.yeo@example.com / password123), an Attendee
-4. Type /events/&lt;reference from step 2&gt; after the site address in the browser address bar (e.g. http://localhost:3000/events/&lt;reference from step 2&gt;) and press Enter</t>
+          <t>1. Click 'My Registrations' in the sidebar
+2. Click 'SPM51 Sold Out Summit'</t>
         </is>
       </c>
     </row>
@@ -1563,11 +1564,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM51 Private Board Dinner (Confirmed, registration off) | Attendee: Marcus Yeo</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Attendee: Jocelyn Pang | SPM51 Last Seat Masterclass: registered | SPM51 Sold Out Summit: waitlisted</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="112" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1575,8 +1576,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The event page shows the 'Confirmed' status badge and 'Registration: Not enabled for this event'.
-Step 4: The page shows 'This event doesn't exist, or you don't have access to it.' and nothing about registering.</t>
+          <t>Step 1: The 'My Registrations' page opens with a table of Event, When and Status. 'SPM51 Last Seat Masterclass' (22 Jan 2028, 09:00–17:00) shows the badge 'Registered', and 'SPM51 Sold Out Summit' (29 Jan 2028, 09:00–17:00) shows 'Waiting list'.
+Step 2: The 'SPM51 Sold Out Summit' event page opens. The 'Your registration' card shows the 'Waiting list' badge and 'You're on the waiting list.', with no 'Register' button.</t>
         </is>
       </c>
     </row>
@@ -1685,11 +1686,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC11</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="139" customHeight="1">
+          <t>SPM-51-TC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="98.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1698,12 +1699,12 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Test data loaded: `npm run fixtures:spm51` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM51 …' events, never anyone else's data).
-Logged in as Jocelyn Pang (jocelyn.pang@example.com / password123), an Attendee registered for 'SPM51 Last Seat Masterclass' and on the waiting list for 'SPM51 Sold Out Summit'. (The base seed may register her for other events too; those rows are listed as well.)
-Nothing is saved in this case.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="31" customHeight="1">
+Nothing is saved in this case.
+Start logged in as Daniel Tan (daniel.tan@connectsphere.com / password123), a coordinator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="139" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1711,8 +1712,11 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'My Registrations' in the sidebar
-2. Click 'SPM51 Sold Out Summit'</t>
+          <t>1. Type /browse after the site address in the browser address bar (e.g. http://localhost:3000/browse) and press Enter
+2. Type /registrations after the site address in the browser address bar and press Enter
+3. Click 'All Events' in the sidebar and open 'SPM51 Harbour Open House'
+4. Log out and log in as Evelyn Chen (evelyn.chen@straitsmedic.com / password123), who organised every 'SPM51 …' event
+5. Click 'My Events' in the sidebar and open 'SPM51 Harbour Open House'</t>
         </is>
       </c>
     </row>
@@ -1724,11 +1728,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Attendee: Jocelyn Pang | SPM51 Last Seat Masterclass: registered | SPM51 Sold Out Summit: waitlisted</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="112" customHeight="1">
+          <t>Event: SPM51 Harbour Open House (open for registration) | Users: Daniel Tan (coordinator), Evelyn Chen (organiser)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="152.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1736,8 +1740,10 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The 'My Registrations' page opens with a table of Event, When and Status. 'SPM51 Last Seat Masterclass' (22 Jan 2028, 09:00–17:00) shows the badge 'Registered', and 'SPM51 Sold Out Summit' (29 Jan 2028, 09:00–17:00) shows 'Waiting list'.
-Step 2: The 'SPM51 Sold Out Summit' event page opens. The 'Your registration' card shows the 'Waiting list' badge and 'You're on the waiting list.', with no 'Register' button.</t>
+          <t>Step 1: The 'Browse Events' page shows a red alert 'You do not have access to this' with 'Browsing and registering for events is what an Attendee account is for.' and a 'Back to Dashboard' button. No events are listed.
+Step 2: The 'My Registrations' page shows 'You do not have access to this' with 'Registrations belong to an Attendee account.'
+Step 3: The event page shows the Registration card, but no 'Your registration' card and no 'Register' button.
+Step 5: The event page shows the Registration card, but no 'Your registration' card and no 'Register' button.</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -1846,7 +1852,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC12</t>
+          <t>SPM-51-TC01</t>
         </is>
       </c>
     </row>
@@ -1859,12 +1865,12 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Test data loaded: `npm run fixtures:spm51` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM51 …' events, never anyone else's data).
-Nothing is saved in this case.
-Start logged in as Daniel Tan (daniel.tan@connectsphere.com / password123), a coordinator.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="139" customHeight="1">
+Logged in as Chua Mei Ling (chua.mei.ling@example.com / password123), an Attendee.
+Nothing is saved in this case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1872,11 +1878,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Type /browse after the site address in the browser address bar (e.g. http://localhost:3000/browse) and press Enter
-2. Type /registrations after the site address in the browser address bar and press Enter
-3. Click 'All Events' in the sidebar and open 'SPM51 Harbour Open House'
-4. Log out and log in as Evelyn Chen (evelyn.chen@straitsmedic.com / password123), who organised every 'SPM51 …' event
-5. Click 'My Events' in the sidebar and open 'SPM51 Harbour Open House'</t>
+          <t>1. Click 'Browse Events' in the sidebar</t>
         </is>
       </c>
     </row>
@@ -1888,11 +1890,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM51 Harbour Open House (open for registration) | Users: Daniel Tan (coordinator), Evelyn Chen (organiser)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="152.5" customHeight="1">
+          <t>Attendee: Chua Mei Ling | Today: after 1 Sept 2026 and before 1 Nov 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="125.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1900,10 +1902,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The 'Browse Events' page shows a red alert 'You do not have access to this' with 'Browsing and registering for events is what an Attendee account is for.' and a 'Back to Dashboard' button. No events are listed.
-Step 2: The 'My Registrations' page shows 'You do not have access to this' with 'Registrations belong to an Attendee account.'
-Step 3: The event page shows the Registration card, but no 'Your registration' card and no 'Register' button.
-Step 5: The event page shows the Registration card, but no 'Your registration' card and no 'Register' button.</t>
+          <t>Step 1: The 'Browse Events' page opens. Among the events listed are 'SPM51 Harbour Open House' and 'SPM51 Last Seat Masterclass' with the badge 'Open', 'SPM51 Early Bird Seminar' with 'Opens 1 Nov 2027, 09:00', 'SPM51 Closed Doors Workshop' with 'Closed', 'SPM51 Undated Talk' with 'Dates not set' and 'SPM51 Sold Out Summit' with 'Full'. Each shows its date and time and the company 'Straits Medical Institute'. 'SPM51 Private Board Dinner' (registration off) and 'SPM51 Planning Stage Forum' (not Confirmed) are not listed.</t>
         </is>
       </c>
     </row>
@@ -1980,127 +1979,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="75" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" s="7" t="inlineStr">
-        <is>
-          <t>Question / ambiguity for the PO or developer</t>
-        </is>
-      </c>
-      <c r="C1" s="7" t="inlineStr">
-        <is>
-          <t>Answer</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="58" customHeight="1">
-      <c r="A2" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="11" t="inlineStr">
-        <is>
-          <t>Written before the code (TDD, 2026-10-10). No screen exists yet, so every label, message and page address below was chosen by the team and is what the developer builds to. Decisions are also recorded in DOCUMENTATION.md (changelog 2026-10-10, Sammi Chua, SPM-51).</t>
-        </is>
-      </c>
-      <c r="C2" s="11" t="n"/>
-    </row>
-    <row r="3" ht="85" customHeight="1">
-      <c r="A3" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED 2026-10-10: Browse Events (S-26) is the attendee's 'Browse Events' sidebar link (/browse). It lists every Confirmed event with registration enabled, each with its title, date and time, company and a registration badge: 'Open', 'Opens &lt;date, time&gt;', 'Closed', 'Full' or 'Dates not set'. Each title links to the event page. With none: 'No events are open for registration right now.'</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="n"/>
-    </row>
-    <row r="4" ht="179.5" customHeight="1">
-      <c r="A4" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED 2026-10-10: on the event page an attendee sees, below the read-only Registration card (SPM-64: Registration, Capacity, Opens, Closes), a 'Your registration' card. Open: optional 'Dietary requirements' and 'Accessibility requirements' fields and a 'Register' button; after registering, a green alert 'You're registered for this event.' and the status badge 'Registered'. Already registered: the 'Registered' badge and 'You registered on &lt;date&gt;.'. On the waiting list: the 'Waiting list' badge and 'You're on the waiting list.'. Not yet open: 'Registration opens &lt;date, time&gt;.'. Closed: 'Registration closed on &lt;date, time&gt;.'. No dates: 'Registration dates haven't been set for this event.'. Full: 'This event is full. You can join the waiting list instead.' and 'Joining the waiting list isn't available yet.' No Register button in any of those states.</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n"/>
-    </row>
-    <row r="5" ht="71.5" customHeight="1">
-      <c r="A5" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED 2026-10-10: My Registrations (S-27) is the attendee's 'My Registrations' sidebar link (/registrations): a table of Event (linking to it), When and Status (badge: 'Registered', 'Waiting list', 'Withdrawn', 'Attended'), newest registration first. With none: 'You haven't registered for any events yet.'</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n"/>
-    </row>
-    <row r="6" ht="125.5" customHeight="1">
-      <c r="A6" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>DECIDED 2026-10-10: refusals, as the route already words them, shown in a red alert in the 'Your registration' card: 'Already registered for this event', 'This event is full', 'Registration has not opened yet', 'Registration has closed', 'Registration dates haven't been set for this event', 'Registration is not enabled for this event'. Pages other roles can't use show the existing refusal: 'You do not have access to this' with 'Browsing and registering for events is what an Attendee account is for.' (Browse Events) or 'Registrations belong to an Attendee account.' (My Registrations).</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n"/>
-    </row>
-    <row r="7" ht="71.5" customHeight="1">
-      <c r="A7" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Not reachable from the screens, so covered by unit tests only: the exact opening and closing moments (a tester can't pick the clock), two attendees taking the last seat at the same moment, a non-attendee calling the register API directly, and re-registering after withdrawing (there is no withdraw screen yet).</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="n"/>
-    </row>
-    <row r="8" ht="301" customHeight="1">
-      <c r="A8" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Fixtures needed (scripts/seed-spm51.ts, `npm run fixtures:spm51`, to be written with the code). Every event: organiser Evelyn Chen (Straits Medical Institute), coordinator Daniel Tan, 09:00-17:00. Open period = opens 1 Sept 2026 09:00, closes 31 Dec 2027 17:00.
-- 'SPM51 Harbour Open House': Confirmed, 15 Jan 2028, on, capacity 50, open period, no registrations.
-- 'SPM51 Last Seat Masterclass': Confirmed, 22 Jan 2028, on, capacity 3, open period; Jocelyn Pang and Ravi Subramaniam registered, Bryan Chua withdrawn.
-- 'SPM51 Sold Out Summit': Confirmed, 29 Jan 2028, on, capacity 3, open period; Kavitha Menon, Daniel Lim and Amirah Rashid registered, Jocelyn Pang waitlisted, Wong Kai Xin withdrawn.
-- 'SPM51 Early Bird Seminar': Confirmed, 20 Jan 2028, on, capacity 50, opens 1 Nov 2027 09:00, closes 31 Dec 2027 17:00.
-- 'SPM51 Closed Doors Workshop': Confirmed, 10 Dec 2027, on, capacity 50, opens 1 Aug 2026 09:00, closes 30 Sept 2026 17:00.
-- 'SPM51 Undated Talk': Confirmed, 5 Feb 2028, on, capacity 50, no dates.
-- 'SPM51 Private Board Dinner': Confirmed, 12 Feb 2028, registration off.
-- 'SPM51 Planning Stage Forum': Planning, 19 Feb 2028, on, capacity 50, open period.</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -2133,11 +2011,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC01</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="98.5" customHeight="1">
+          <t>SPM-51-TC02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2146,12 +2024,12 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Test data loaded: `npm run fixtures:spm51` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM51 …' events, never anyone else's data).
-Logged in as Chua Mei Ling (chua.mei.ling@example.com / password123), an Attendee.
-Nothing is saved in this case.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="17.5" customHeight="1">
+Before and after: run `npm run fixtures:spm51` (never `npx prisma db seed`, which wipes everyone's data).
+Logged in as Chua Mei Ling (chua.mei.ling@example.com / password123), an Attendee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="71.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2159,11 +2037,15 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Browse Events' in the sidebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+          <t>1. Click 'Browse Events' in the sidebar
+2. Click 'SPM51 Harbour Open House'
+3. Enter 'Vegetarian' in 'Dietary requirements'
+4. Click 'Register'
+5. Reload the page</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2171,11 +2053,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Attendee: Chua Mei Ling | Today: after 1 Sept 2026 and before 1 Nov 2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="125.5" customHeight="1">
+          <t>Event: SPM51 Harbour Open House (Confirmed, capacity 50, open 1 Sept 2026 09:00 to 31 Dec 2027 17:00) | Dietary requirements: Vegetarian</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="152.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2183,7 +2065,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The 'Browse Events' page opens. Among the events listed are 'SPM51 Harbour Open House' and 'SPM51 Last Seat Masterclass' with the badge 'Open', 'SPM51 Early Bird Seminar' with 'Opens 1 Nov 2027, 09:00', 'SPM51 Closed Doors Workshop' with 'Closed', 'SPM51 Undated Talk' with 'Dates not set' and 'SPM51 Sold Out Summit' with 'Full'. Each shows its date and time and the company 'Straits Medical Institute'. 'SPM51 Private Board Dinner' (registration off) and 'SPM51 Planning Stage Forum' (not Confirmed) are not listed.</t>
+          <t>Step 2: The event page opens. The Registration card shows 'Registration: Enabled', 'Capacity: 50', 'Opens: 1 Sept 2026, 09:00' and 'Closes: 31 Dec 2027, 17:00'. The 'Your registration' card shows the optional fields 'Dietary requirements' and 'Accessibility requirements' and a 'Register' button.
+Step 4: A green alert 'You're registered for this event.' appears, with the status badge 'Registered'. The Register button is gone.
+Step 5: The 'Your registration' card still shows the 'Registered' badge and 'You registered on &lt;today's date&gt;.', with no Register button.</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2176,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC02</t>
+          <t>SPM-51-TC03</t>
         </is>
       </c>
     </row>
@@ -2306,11 +2190,11 @@
         <is>
           <t>Test data loaded: `npm run fixtures:spm51` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM51 …' events, never anyone else's data).
 Before and after: run `npm run fixtures:spm51` (never `npx prisma db seed`, which wipes everyone's data).
-Logged in as Chua Mei Ling (chua.mei.ling@example.com / password123), an Attendee.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="71.5" customHeight="1">
+Logged in as Tan Jia Hui (tan.jia.hui@example.com / password123), an Attendee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2318,15 +2202,15 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Browse Events' in the sidebar
-2. Click 'SPM51 Harbour Open House'
-3. Enter 'Vegetarian' in 'Dietary requirements'
-4. Click 'Register'
-5. Reload the page</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
+          <t>1. Click 'Browse Events' in the sidebar and open 'SPM51 Harbour Open House'
+2. Open the same page in a second browser tab
+3. In the first tab, click 'Register'
+4. In the second tab, click 'Register'
+5. Reload the second tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2334,11 +2218,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM51 Harbour Open House (Confirmed, capacity 50, open 1 Sept 2026 09:00 to 31 Dec 2027 17:00) | Dietary requirements: Vegetarian</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="152.5" customHeight="1">
+          <t>Event: SPM51 Harbour Open House | Attendee: Tan Jia Hui | Two tabs open on the same event page before either registers</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2346,9 +2230,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 2: The event page opens. The Registration card shows 'Registration: Enabled', 'Capacity: 50', 'Opens: 1 Sept 2026, 09:00' and 'Closes: 31 Dec 2027, 17:00'. The 'Your registration' card shows the optional fields 'Dietary requirements' and 'Accessibility requirements' and a 'Register' button.
-Step 4: A green alert 'You're registered for this event.' appears, with the status badge 'Registered'. The Register button is gone.
-Step 5: The 'Your registration' card still shows the 'Registered' badge and 'You registered on &lt;today's date&gt;.', with no Register button.</t>
+          <t>Step 3: The first tab shows 'You're registered for this event.' and the 'Registered' badge.
+Step 4: The second tab shows a red alert 'Already registered for this event' in the 'Your registration' card, and no second registration is made.
+Step 5: The second tab now shows the 'Registered' badge and no Register button.</t>
         </is>
       </c>
     </row>
@@ -2457,11 +2341,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC03</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="112" customHeight="1">
+          <t>SPM-51-TC04</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2470,12 +2354,12 @@
       <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Test data loaded: `npm run fixtures:spm51` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM51 …' events, never anyone else's data).
-Before and after: run `npm run fixtures:spm51` (never `npx prisma db seed`, which wipes everyone's data).
-Logged in as Tan Jia Hui (tan.jia.hui@example.com / password123), an Attendee.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
+Before: run `npm run fixtures:spm51`. After: go straight to SPM-51-TC05, which checks the full event, and reset after it.
+Logged in as Tom Harris (tom.harris@example.com / password123), an Attendee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2483,11 +2367,8 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Browse Events' in the sidebar and open 'SPM51 Harbour Open House'
-2. Open the same page in a second browser tab
-3. In the first tab, click 'Register'
-4. In the second tab, click 'Register'
-5. Reload the second tab</t>
+          <t>1. Click 'Browse Events' in the sidebar and open 'SPM51 Last Seat Masterclass'
+2. Click 'Register'</t>
         </is>
       </c>
     </row>
@@ -2499,11 +2380,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM51 Harbour Open House | Attendee: Tan Jia Hui | Two tabs open on the same event page before either registers</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
+          <t>Event: SPM51 Last Seat Masterclass (capacity 3; 2 registered, 1 withdrawn) | Attendee: Tom Harris</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2511,9 +2392,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 3: The first tab shows 'You're registered for this event.' and the 'Registered' badge.
-Step 4: The second tab shows a red alert 'Already registered for this event' in the 'Your registration' card, and no second registration is made.
-Step 5: The second tab now shows the 'Registered' badge and no Register button.</t>
+          <t>Step 1: The Registration card shows 'Capacity: 3', and the 'Your registration' card shows a 'Register' button: the withdrawn attendee doesn't hold a seat.
+Step 2: 'You're registered for this event.' appears with the 'Registered' badge. Tom Harris has the third and last seat.</t>
         </is>
       </c>
     </row>
@@ -2622,11 +2502,11 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC04</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="125.5" customHeight="1">
+          <t>SPM-51-TC05</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="98.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2634,13 +2514,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Test data loaded: `npm run fixtures:spm51` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM51 …' events, never anyone else's data).
-Before: run `npm run fixtures:spm51`. After: go straight to SPM-51-TC05, which checks the full event, and reset after it.
-Logged in as Tom Harris (tom.harris@example.com / password123), an Attendee.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
+          <t>SPM-51-TC04 has just been run (SPM51 Last Seat Masterclass now has 3 of 3 seats taken).
+After: run `npm run fixtures:spm51` (never `npx prisma db seed`, which wipes everyone's data).
+Log out, then log in as Farhan Ismail (farhan.ismail@example.com / password123), an Attendee with no registration for this event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="31" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2648,8 +2528,8 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Browse Events' in the sidebar and open 'SPM51 Last Seat Masterclass'
-2. Click 'Register'</t>
+          <t>1. Click 'Browse Events' in the sidebar
+2. Click 'SPM51 Last Seat Masterclass'</t>
         </is>
       </c>
     </row>
@@ -2661,11 +2541,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM51 Last Seat Masterclass (capacity 3; 2 registered, 1 withdrawn) | Attendee: Tom Harris</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Event: SPM51 Last Seat Masterclass (capacity 3, now 3 registered) | Attendee: Farhan Ismail</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="85" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2673,8 +2553,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The Registration card shows 'Capacity: 3', and the 'Your registration' card shows a 'Register' button: the withdrawn attendee doesn't hold a seat.
-Step 2: 'You're registered for this event.' appears with the 'Registered' badge. Tom Harris has the third and last seat.</t>
+          <t>Step 1: 'SPM51 Last Seat Masterclass' now has the badge 'Full'.
+Step 2: The 'Your registration' card shows 'This event is full. You can join the waiting list instead.' and 'Joining the waiting list isn't available yet.' There is no 'Register' button.</t>
         </is>
       </c>
     </row>
@@ -2783,7 +2663,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC05</t>
+          <t>SPM-51-TC06</t>
         </is>
       </c>
     </row>
@@ -2795,9 +2675,9 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC04 has just been run (SPM51 Last Seat Masterclass now has 3 of 3 seats taken).
-After: run `npm run fixtures:spm51` (never `npx prisma db seed`, which wipes everyone's data).
-Log out, then log in as Farhan Ismail (farhan.ismail@example.com / password123), an Attendee with no registration for this event.</t>
+          <t>Test data loaded: `npm run fixtures:spm51` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM51 …' events, never anyone else's data).
+Logged in as Chua Mei Ling (chua.mei.ling@example.com / password123), an Attendee.
+Nothing is saved in this case.</t>
         </is>
       </c>
     </row>
@@ -2809,12 +2689,11 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Browse Events' in the sidebar
-2. Click 'SPM51 Last Seat Masterclass'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+          <t>1. Click 'Browse Events' in the sidebar and open 'SPM51 Early Bird Seminar'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2822,11 +2701,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM51 Last Seat Masterclass (capacity 3, now 3 registered) | Attendee: Farhan Ismail</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
+          <t>Event: SPM51 Early Bird Seminar (registration opens 1 Nov 2027, 09:00, closes 31 Dec 2027, 17:00) | Today: before 1 Nov 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2834,8 +2713,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: 'SPM51 Last Seat Masterclass' now has the badge 'Full'.
-Step 2: The 'Your registration' card shows 'This event is full. You can join the waiting list instead.' and 'Joining the waiting list isn't available yet.' There is no 'Register' button.</t>
+          <t>Step 1: The Registration card shows 'Opens: 1 Nov 2027, 09:00' and 'Closes: 31 Dec 2027, 17:00'. The 'Your registration' card says 'Registration opens 1 Nov 2027, 09:00.' and has no 'Register' button.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2822,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC06</t>
+          <t>SPM-51-TC07</t>
         </is>
       </c>
     </row>
@@ -2970,11 +2848,11 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Browse Events' in the sidebar and open 'SPM51 Early Bird Seminar'</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
+          <t>1. Click 'Browse Events' in the sidebar and open 'SPM51 Closed Doors Workshop'</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2982,7 +2860,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM51 Early Bird Seminar (registration opens 1 Nov 2027, 09:00, closes 31 Dec 2027, 17:00) | Today: before 1 Nov 2027</t>
+          <t>Event: SPM51 Closed Doors Workshop (registration 1 Aug 2026, 09:00 to 30 Sept 2026, 17:00) | Today: after 30 Sept 2026</t>
         </is>
       </c>
     </row>
@@ -2994,7 +2872,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The Registration card shows 'Opens: 1 Nov 2027, 09:00' and 'Closes: 31 Dec 2027, 17:00'. The 'Your registration' card says 'Registration opens 1 Nov 2027, 09:00.' and has no 'Register' button.</t>
+          <t>Step 1: The Registration card shows 'Opens: 1 Aug 2026, 09:00' and 'Closes: 30 Sept 2026, 17:00'. The 'Your registration' card says 'Registration closed on 30 Sept 2026, 17:00.' and has no 'Register' button.</t>
         </is>
       </c>
     </row>
@@ -3103,7 +2981,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>SPM-51-TC07</t>
+          <t>SPM-51-TC08</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3007,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Browse Events' in the sidebar and open 'SPM51 Closed Doors Workshop'</t>
+          <t>1. Click 'Browse Events' in the sidebar and open 'SPM51 Undated Talk'</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3019,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM51 Closed Doors Workshop (registration 1 Aug 2026, 09:00 to 30 Sept 2026, 17:00) | Today: after 30 Sept 2026</t>
+          <t>Event: SPM51 Undated Talk (Confirmed, registration on, capacity 50, no opening or closing date)</t>
         </is>
       </c>
     </row>
@@ -3153,7 +3031,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The Registration card shows 'Opens: 1 Aug 2026, 09:00' and 'Closes: 30 Sept 2026, 17:00'. The 'Your registration' card says 'Registration closed on 30 Sept 2026, 17:00.' and has no 'Register' button.</t>
+          <t>Step 1: The Registration card shows 'Opens: —' and 'Closes: —'. The 'Your registration' card says 'Registration dates haven't been set for this event.' and has no 'Register' button.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Browse Events and each event's registration state
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-51_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-51_Test_Cases.xlsx
@@ -1894,7 +1894,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="125.5" customHeight="1">
+    <row r="6" ht="139" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: The 'Browse Events' page opens. Among the events listed are 'SPM51 Harbour Open House' and 'SPM51 Last Seat Masterclass' with the badge 'Open', 'SPM51 Early Bird Seminar' with 'Opens 1 Nov 2027, 09:00', 'SPM51 Closed Doors Workshop' with 'Closed', 'SPM51 Undated Talk' with 'Dates not set' and 'SPM51 Sold Out Summit' with 'Full'. Each shows its date and time and the company 'Straits Medical Institute'. 'SPM51 Private Board Dinner' (registration off) and 'SPM51 Planning Stage Forum' (not Confirmed) are not listed.</t>
+          <t>Step 1: The 'Browse Events' page opens. Among the events listed are 'SPM51 Harbour Open House' and 'SPM51 Last Seat Masterclass' with the badge 'Open', 'SPM51 Early Bird Seminar' with 'Not open yet' and 'Opens 1 Nov 2027, 09:00' beside it, 'SPM51 Closed Doors Workshop' with 'Closed', 'SPM51 Undated Talk' with 'Dates not set' and 'SPM51 Sold Out Summit' with 'Full'. Each shows its date and time and the company 'Straits Medical Institute'. 'SPM51 Private Board Dinner' (registration off) and 'SPM51 Planning Stage Forum' (not Confirmed) are not listed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-51 Fixtures, docs and test cases re-checked
- npm run fixtures:spm51 (scripts/seed-spm51.ts): the 8 "SPM51 ..." events
  with their registration settings and registrations; mirrored at the end
  of prisma/seed.ts
- Test cases: code_references filled in; server side of every case run
  against the fixtures through the API (21 checks as expected)
- DOCUMENTATION.md: eligibility business rule, fixtures command, Known Gaps
  (Browse Events row closed; waiting-list joining and withdraw #20 added)
- docs/PERMISSIONS.md: GET /api/registrations, eligibility on POST
- UI_DESIGN.md: S-26, S-27 and the "Your registration" card

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-51_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-51_Test_Cases.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1126,8 +1126,34 @@
       </c>
       <c r="F28" s="9" t="n"/>
     </row>
+    <row r="30" ht="152.5" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Code reviewed</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>src/lib/registrationEligibility.ts
+src/app/api/registrations/route.ts
+src/app/api/events/route.ts
+src/app/api/events/[id]/route.ts
+src/lib/permissions.ts
+src/lib/statuses.ts
+src/app/browse/page.tsx
+src/app/events/[id]/RegisterPanel.tsx
+src/app/events/[id]/page.tsx
+src/app/registrations/page.tsx
+scripts/seed-spm51.ts</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="9" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="24">
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="E24:F24"/>
     <mergeCell ref="E23:F23"/>
@@ -1143,6 +1169,7 @@
     <mergeCell ref="E27:F27"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B30:F30"/>
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B18:D18"/>

</xml_diff>

<commit_message>
SPM-66: Update BPMN, clarifications and affected test cases
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-51_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-51_Test_Cases.xlsx
@@ -136,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -182,6 +182,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -726,11 +729,15 @@
       </c>
       <c r="G8" s="24" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="H8" s="24" t="n"/>
-      <c r="I8" s="24" t="n"/>
+      <c r="I8" s="24" t="inlineStr">
+        <is>
+          <t>#26</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="12" customHeight="1" s="20">
       <c r="A9" s="5" t="inlineStr">
@@ -960,11 +967,15 @@
       </c>
       <c r="G14" s="24" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="H14" s="24" t="n"/>
-      <c r="I14" s="24" t="n"/>
+      <c r="I14" s="24" t="inlineStr">
+        <is>
+          <t>#26</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12" customHeight="1" s="20">
       <c r="A15" s="5" t="inlineStr">
@@ -4769,7 +4780,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="24.88" customWidth="1" style="20" min="1" max="1"/>
@@ -4777,45 +4788,52 @@
     <col width="12.63" customWidth="1" style="20" min="3" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="20">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="90" customHeight="1" s="20">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>v2 (2026-10-27): A waiting attendee's 'Your registration' card now reads 'You're number 1 on the waiting list.' (not 'You're on the waiting list.') and has a 'Leave waiting list' button; My Registrations also shows 'Number 1 in the queue' under the 'Waiting list' badge (SPM-66 AC3 and AC4: the Attendee sees their position and can leave the list). Read the expected result with the new wording. The behaviour this case checks is unchanged. (Step 2: still no 'Register' button.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" s="20">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="9" t="n"/>
-    </row>
-    <row r="2" ht="17.25" customHeight="1" s="20">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="B2" s="9" t="n"/>
+    </row>
+    <row r="3" ht="17.25" customHeight="1" s="20">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>SPM-51-TC11</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30.75" customHeight="1" s="20">
-      <c r="A3" s="10" t="inlineStr">
+    <row r="4" ht="30.75" customHeight="1" s="20">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>My Registrations lists the attendee's registrations with their status</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="138.75" customHeight="1" s="20">
-      <c r="A4" s="10" t="inlineStr">
+    <row r="5" ht="138.75" customHeight="1" s="20">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Test data loaded: `npm run fixtures:spm51` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM51 …' events, never anyone else's data).
 Logged in as Jocelyn Pang (jocelyn.pang@example.com / password123), an Attendee registered for 'SPM51 Last Seat Masterclass' and on the waiting list for 'SPM51 Sold Out Summit'. (The base seed may register her for other events too; those rows are listed as well.)
@@ -4823,204 +4841,203 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30.75" customHeight="1" s="20">
-      <c r="A5" s="10" t="inlineStr">
+    <row r="6" ht="30.75" customHeight="1" s="20">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>1. Click 'My Registrations' in the sidebar
 2. Click 'SPM51 Sold Out Summit'</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30.75" customHeight="1" s="20">
-      <c r="A6" s="10" t="inlineStr">
+    <row r="7" ht="30.75" customHeight="1" s="20">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Attendee: Jocelyn Pang | SPM51 Last Seat Masterclass: registered | SPM51 Sold Out Summit: waitlisted</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="111.75" customHeight="1" s="20">
-      <c r="A7" s="10" t="inlineStr">
+    <row r="8" ht="111.75" customHeight="1" s="20">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Step 1: The 'My Registrations' page opens with a table of Event, When and Status. 'SPM51 Last Seat Masterclass' (22 Jan 2028, 09:00–17:00) shows the badge 'Registered', and 'SPM51 Sold Out Summit' (29 Jan 2028, 09:00–17:00) shows 'Waiting list'.
 Step 2: The 'SPM51 Sold Out Summit' event page opens. The 'Your registration' card shows the 'Waiting list' badge and 'You're on the waiting list.', with no 'Register' button.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="17.25" customHeight="1" s="20">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="9" ht="17.25" customHeight="1" s="20">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" s="20">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="10" ht="15.75" customHeight="1" s="20">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B10" s="11" t="n">
         <v>46307</v>
       </c>
     </row>
-    <row r="10" ht="15.75" customHeight="1" s="20"/>
-    <row r="11" ht="15.75" customHeight="1" s="20">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="11" ht="15.75" customHeight="1" s="20"/>
+    <row r="12" ht="15.75" customHeight="1" s="20">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="14" t="n"/>
-    </row>
-    <row r="12" ht="15.75" customHeight="1" s="20">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="14" t="n"/>
+    </row>
+    <row r="13" ht="15.75" customHeight="1" s="20">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Step 1: The 'My Registrations' page opens with a table of Event, When and Status. 'SPM51 Last Seat Masterclass' (22 Jan 2028, 09:00–17:00) shows the badge 'Registered', and 'SPM51 Sold Out Summit' (29 Jan 2028, 09:00–17:00) shows 'Waiting list'.
 Step 2: The 'SPM51 Sold Out Summit' event page opens. The 'Your registration' card shows the 'Waiting list' badge and 'You're on the waiting list.', with no 'Register' button.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1" s="20">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
     <row r="14" ht="15.75" customHeight="1" s="20">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="20">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>Sammi</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="20">
       <c r="A16" s="18" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15.75" customHeight="1" s="20">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B17" s="19" t="n">
         <v>46308</v>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="20"/>
-    <row r="18" ht="15.75" customHeight="1" s="20">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="18" ht="15.75" customHeight="1" s="20"/>
+    <row r="19" ht="15.75" customHeight="1" s="20">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n"/>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" s="20">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="B19" s="13" t="n"/>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" s="20">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Step 1: The 'My Registrations' page opens with a table of Event, When and Status. 'SPM51 Last Seat Masterclass' (22 Jan 2028, 09:00–17:00) shows the badge 'Registered', and 'SPM51 Sold Out Summit' (29 Jan 2028, 09:00–17:00) shows 'Waiting list'.
 Step 2: The 'SPM51 Sold Out Summit' event page opens. The 'Your registration' card shows the 'Waiting list' badge and 'You're on the waiting list.', with no 'Register' button.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1" s="20">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
     <row r="21" ht="15.75" customHeight="1" s="20">
       <c r="A21" s="18" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="20">
       <c r="A22" s="18" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B22" s="18" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="20">
       <c r="A23" s="18" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Kristen</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="20">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B23" s="19" t="n">
+      <c r="B24" s="19" t="n">
         <v>46308</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="20"/>
     <row r="25" ht="15.75" customHeight="1" s="20"/>
     <row r="26" ht="15.75" customHeight="1" s="20"/>
     <row r="27" ht="15.75" customHeight="1" s="20"/>
@@ -5997,7 +6014,11 @@
     <row r="998" ht="15.75" customHeight="1" s="20"/>
     <row r="999" ht="15.75" customHeight="1" s="20"/>
     <row r="1000" ht="15.75" customHeight="1" s="20"/>
+    <row r="1001" ht="15.75" customHeight="1" s="20"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
@@ -12226,7 +12247,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="24.88" customWidth="1" style="20" min="1" max="1"/>
@@ -12234,45 +12255,52 @@
     <col width="12.63" customWidth="1" style="20" min="3" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="20">
-      <c r="A1" s="8" t="inlineStr">
+    <row r="1" ht="90" customHeight="1" s="20">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>v2 (2026-10-27): A full event's 'Your registration' card now has a 'Join waiting list' button, with the optional Dietary requirements and Accessibility requirements fields, under 'This event is full. You can join the waiting list instead.' It no longer says 'Joining the waiting list isn't available yet.' (SPM-66 AC1: an Attendee can join the waiting list of a full event). Read step 2's expected result with the new card. There is still no 'Register' button, so the behaviour this case checks is unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" s="20">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="9" t="n"/>
-    </row>
-    <row r="2" ht="17.25" customHeight="1" s="20">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="B2" s="9" t="n"/>
+    </row>
+    <row r="3" ht="17.25" customHeight="1" s="20">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>SPM-51-TC05</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30.75" customHeight="1" s="20">
-      <c r="A3" s="10" t="inlineStr">
+    <row r="4" ht="30.75" customHeight="1" s="20">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Once the capacity is reached, registration is refused and the waiting list is offered instead</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="98.25" customHeight="1" s="20">
-      <c r="A4" s="10" t="inlineStr">
+    <row r="5" ht="98.25" customHeight="1" s="20">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>SPM-51-TC04 has just been run (SPM51 Last Seat Masterclass now has 3 of 3 seats taken).
 After: run `npm run fixtures:spm51` (never `npx prisma db seed`, which wipes everyone's data).
@@ -12280,204 +12308,203 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30.75" customHeight="1" s="20">
-      <c r="A5" s="10" t="inlineStr">
+    <row r="6" ht="30.75" customHeight="1" s="20">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>1. Click 'Browse Events' in the sidebar
 2. Click 'SPM51 Last Seat Masterclass'</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30.75" customHeight="1" s="20">
-      <c r="A6" s="10" t="inlineStr">
+    <row r="7" ht="30.75" customHeight="1" s="20">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Event: SPM51 Last Seat Masterclass (capacity 3, now 3 registered) | Attendee: Farhan Ismail</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="84.75" customHeight="1" s="20">
-      <c r="A7" s="10" t="inlineStr">
+    <row r="8" ht="84.75" customHeight="1" s="20">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Step 1: 'SPM51 Last Seat Masterclass' now has the badge 'Full'.
 Step 2: The 'Your registration' card shows 'This event is full. You can join the waiting list instead.' and 'Joining the waiting list isn't available yet.' There is no 'Register' button.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="17.25" customHeight="1" s="20">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="9" ht="17.25" customHeight="1" s="20">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" s="20">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="10" ht="15.75" customHeight="1" s="20">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B10" s="11" t="n">
         <v>46307</v>
       </c>
     </row>
-    <row r="10" ht="15.75" customHeight="1" s="20"/>
-    <row r="11" ht="15.75" customHeight="1" s="20">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="11" ht="15.75" customHeight="1" s="20"/>
+    <row r="12" ht="15.75" customHeight="1" s="20">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="14" t="n"/>
-    </row>
-    <row r="12" ht="15.75" customHeight="1" s="20">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="14" t="n"/>
+    </row>
+    <row r="13" ht="15.75" customHeight="1" s="20">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Step 1: 'SPM51 Last Seat Masterclass' now has the badge 'Full'.
 Step 2: The 'Your registration' card shows 'This event is full. You can join the waiting list instead.' and 'Joining the waiting list isn't available yet.' There is no 'Register' button.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1" s="20">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
     <row r="14" ht="15.75" customHeight="1" s="20">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="20">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>Sammi</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="20">
       <c r="A16" s="18" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15.75" customHeight="1" s="20">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B17" s="19" t="n">
         <v>46308</v>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="20"/>
-    <row r="18" ht="15.75" customHeight="1" s="20">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="18" ht="15.75" customHeight="1" s="20"/>
+    <row r="19" ht="15.75" customHeight="1" s="20">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n"/>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" s="20">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="B19" s="13" t="n"/>
+    </row>
+    <row r="20" ht="15.75" customHeight="1" s="20">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Step 1: 'SPM51 Last Seat Masterclass' now has the badge 'Full'.
 Step 2: The 'Your registration' card shows 'This event is full. You can join the waiting list instead.' and 'Joining the waiting list isn't available yet.' There is no 'Register' button.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1" s="20">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
     <row r="21" ht="15.75" customHeight="1" s="20">
       <c r="A21" s="18" t="inlineStr">
         <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="20">
       <c r="A22" s="18" t="inlineStr">
         <is>
-          <t>Executed by</t>
+          <t>Remarks</t>
         </is>
       </c>
       <c r="B22" s="18" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="20">
       <c r="A23" s="18" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Kristen</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="20">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B23" s="19" t="n">
+      <c r="B24" s="19" t="n">
         <v>46308</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="20"/>
     <row r="25" ht="15.75" customHeight="1" s="20"/>
     <row r="26" ht="15.75" customHeight="1" s="20"/>
     <row r="27" ht="15.75" customHeight="1" s="20"/>
@@ -13454,7 +13481,11 @@
     <row r="998" ht="15.75" customHeight="1" s="20"/>
     <row r="999" ht="15.75" customHeight="1" s="20"/>
     <row r="1000" ht="15.75" customHeight="1" s="20"/>
+    <row r="1001" ht="15.75" customHeight="1" s="20"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>

</xml_diff>